<commit_message>
fix: comments for ra ovs
</commit_message>
<xml_diff>
--- a/samples/ra/26-27/Royal Arch Official Visit Matrix 2026 - 2027 MF V8.2 2509026.xlsx
+++ b/samples/ra/26-27/Royal Arch Official Visit Matrix 2026 - 2027 MF V8.2 2509026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0d99dbe784a36402/Desktop/OV matrix 26-27/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kpturner/github/square_ov/samples/ra/26-27/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="8_{170089A2-6D72-4D47-849B-1DB3E2544F59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{11F25216-84EE-4E99-AC65-F8689F0FDA77}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B9FE6B76-02B1-EE4C-AD29-0088D4413930}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{FA0C5B21-D744-41D8-A854-64181BC35FE8}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="48400" windowHeight="24840" tabRatio="500" xr2:uid="{FA0C5B21-D744-41D8-A854-64181BC35FE8}"/>
   </bookViews>
   <sheets>
     <sheet name="2026-2027 Official Visits" sheetId="1" r:id="rId1"/>
@@ -1810,7 +1810,7 @@
     <t>n.sharifi@yahoo.co.uk</t>
   </si>
   <si>
-    <t>CANCELED</t>
+    <t>CANCELLED</t>
   </si>
 </sst>
 </file>
@@ -1820,7 +1820,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="53">
+  <fonts count="53" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -3708,10 +3708,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -4068,35 +4064,35 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DB79890-1B6A-478F-90B1-31B9622852F5}">
   <dimension ref="A1:AZ62"/>
-  <sheetFormatPr defaultColWidth="8" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="46.42578125" style="12" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.140625" style="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.42578125" style="12" customWidth="1"/>
-    <col min="4" max="4" width="18.42578125" style="12" customWidth="1"/>
-    <col min="5" max="5" width="14.42578125" style="29" customWidth="1"/>
-    <col min="6" max="6" width="14.140625" style="12" customWidth="1"/>
-    <col min="7" max="16" width="14.140625" style="14" customWidth="1"/>
-    <col min="17" max="17" width="16.28515625" style="14" customWidth="1"/>
-    <col min="18" max="21" width="14.140625" style="14" customWidth="1"/>
-    <col min="22" max="22" width="13.140625" style="14" customWidth="1"/>
-    <col min="23" max="23" width="14.140625" style="14" customWidth="1"/>
-    <col min="24" max="24" width="14.140625" style="12" customWidth="1"/>
-    <col min="25" max="30" width="14.140625" style="14" customWidth="1"/>
-    <col min="31" max="31" width="15.85546875" style="14" customWidth="1"/>
-    <col min="32" max="37" width="14.140625" style="14" customWidth="1"/>
-    <col min="38" max="40" width="14.140625" style="12" customWidth="1"/>
-    <col min="41" max="41" width="20.140625" style="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="46.5" style="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.1640625" style="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5" style="12" customWidth="1"/>
+    <col min="4" max="4" width="18.5" style="12" customWidth="1"/>
+    <col min="5" max="5" width="14.5" style="29" customWidth="1"/>
+    <col min="6" max="6" width="14.1640625" style="12" customWidth="1"/>
+    <col min="7" max="16" width="14.1640625" style="14" customWidth="1"/>
+    <col min="17" max="17" width="16.33203125" style="14" customWidth="1"/>
+    <col min="18" max="21" width="14.1640625" style="14" customWidth="1"/>
+    <col min="22" max="22" width="13.1640625" style="14" customWidth="1"/>
+    <col min="23" max="23" width="14.1640625" style="14" customWidth="1"/>
+    <col min="24" max="24" width="14.1640625" style="12" customWidth="1"/>
+    <col min="25" max="30" width="14.1640625" style="14" customWidth="1"/>
+    <col min="31" max="31" width="15.83203125" style="14" customWidth="1"/>
+    <col min="32" max="37" width="14.1640625" style="14" customWidth="1"/>
+    <col min="38" max="40" width="14.1640625" style="12" customWidth="1"/>
+    <col min="41" max="41" width="20.1640625" style="12" bestFit="1" customWidth="1"/>
     <col min="42" max="16384" width="8" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:52" ht="15" customHeight="1">
+    <row r="1" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="H1" s="14" t="s">
         <v>558</v>
       </c>
       <c r="V1" s="15"/>
     </row>
-    <row r="2" spans="1:52">
+    <row r="2" spans="1:52" ht="14" x14ac:dyDescent="0.15">
       <c r="E2" s="13" t="s">
         <v>117</v>
       </c>
@@ -4203,7 +4199,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:52" s="15" customFormat="1" ht="60.75" customHeight="1">
+    <row r="3" spans="1:52" s="15" customFormat="1" ht="60.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="E3" s="40" t="s">
         <v>0</v>
       </c>
@@ -4311,7 +4307,7 @@
       </c>
       <c r="AY3" s="12"/>
     </row>
-    <row r="4" spans="1:52" ht="15" customHeight="1">
+    <row r="4" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="C4" s="131" t="s">
         <v>15</v>
       </c>
@@ -4421,7 +4417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:52">
+    <row r="5" spans="1:52" ht="14" x14ac:dyDescent="0.15">
       <c r="C5" s="130" t="s">
         <v>17</v>
       </c>
@@ -4531,7 +4527,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:52">
+    <row r="6" spans="1:52" x14ac:dyDescent="0.2">
       <c r="A6" s="11"/>
       <c r="C6" s="134" t="s">
         <v>18</v>
@@ -4551,14 +4547,14 @@
       <c r="I6" s="107">
         <v>46286</v>
       </c>
-      <c r="J6" s="108" t="s">
-        <v>569</v>
+      <c r="J6" s="108">
+        <v>46289</v>
       </c>
       <c r="K6" s="109">
         <v>46295</v>
       </c>
-      <c r="L6" s="107" t="s">
-        <v>569</v>
+      <c r="L6" s="107">
+        <v>46296</v>
       </c>
       <c r="M6" s="108">
         <v>46304</v>
@@ -4642,7 +4638,7 @@
         <v>46550</v>
       </c>
     </row>
-    <row r="7" spans="1:52" ht="15" customHeight="1">
+    <row r="7" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="C7" s="140" t="s">
         <v>26</v>
       </c>
@@ -4783,7 +4779,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:52" ht="15" customHeight="1">
+    <row r="8" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="C8" s="87" t="s">
         <v>27</v>
       </c>
@@ -4893,7 +4889,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:52" ht="15" customHeight="1">
+    <row r="9" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="E9" s="44" t="s">
         <v>118</v>
       </c>
@@ -4901,9 +4897,13 @@
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
       <c r="I9" s="16"/>
-      <c r="J9" s="16"/>
+      <c r="J9" s="16" t="s">
+        <v>569</v>
+      </c>
       <c r="K9" s="17"/>
-      <c r="L9" s="16"/>
+      <c r="L9" s="16" t="s">
+        <v>569</v>
+      </c>
       <c r="M9" s="16"/>
       <c r="N9" s="16"/>
       <c r="O9" s="8"/>
@@ -4931,7 +4931,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="10" spans="1:52" s="20" customFormat="1">
+    <row r="10" spans="1:52" s="20" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="34" t="s">
         <v>14</v>
       </c>
@@ -5008,7 +5008,7 @@
       </c>
       <c r="AZ10" s="12"/>
     </row>
-    <row r="11" spans="1:52" s="20" customFormat="1">
+    <row r="11" spans="1:52" s="20" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="31" t="s">
         <v>220</v>
       </c>
@@ -5089,7 +5089,7 @@
       </c>
       <c r="AZ11" s="12"/>
     </row>
-    <row r="12" spans="1:52" s="20" customFormat="1">
+    <row r="12" spans="1:52" s="20" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A12" s="19" t="s">
         <v>33</v>
       </c>
@@ -5176,7 +5176,7 @@
       </c>
       <c r="AZ12" s="12"/>
     </row>
-    <row r="13" spans="1:52" s="20" customFormat="1">
+    <row r="13" spans="1:52" s="20" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A13" s="19" t="s">
         <v>34</v>
       </c>
@@ -5263,7 +5263,7 @@
       </c>
       <c r="AZ13" s="12"/>
     </row>
-    <row r="14" spans="1:52">
+    <row r="14" spans="1:52" ht="14" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>35</v>
       </c>
@@ -5349,7 +5349,7 @@
         <v>Simon Edward Banham</v>
       </c>
     </row>
-    <row r="15" spans="1:52">
+    <row r="15" spans="1:52" ht="14" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>41</v>
       </c>
@@ -5435,7 +5435,7 @@
         <v>David Leslie Ryan</v>
       </c>
     </row>
-    <row r="16" spans="1:52" ht="15.75" thickBot="1">
+    <row r="16" spans="1:52" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>46</v>
       </c>
@@ -5553,7 +5553,7 @@
         <v>John Donoghue</v>
       </c>
     </row>
-    <row r="17" spans="1:41" ht="16.5" thickTop="1" thickBot="1">
+    <row r="17" spans="1:41" ht="16" thickTop="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
         <v>48</v>
       </c>
@@ -5641,7 +5641,7 @@
         <v>Anthony John Denton</v>
       </c>
     </row>
-    <row r="18" spans="1:41" ht="15.75" thickTop="1">
+    <row r="18" spans="1:41" thickTop="1" x14ac:dyDescent="0.15">
       <c r="A18" s="3" t="s">
         <v>52</v>
       </c>
@@ -5726,7 +5726,7 @@
         <v>Ronald John Griffiths</v>
       </c>
     </row>
-    <row r="19" spans="1:41">
+    <row r="19" spans="1:41" ht="14" x14ac:dyDescent="0.15">
       <c r="A19" s="3" t="s">
         <v>55</v>
       </c>
@@ -5806,7 +5806,7 @@
         <v>Michael John Ingram</v>
       </c>
     </row>
-    <row r="20" spans="1:41">
+    <row r="20" spans="1:41" ht="14" x14ac:dyDescent="0.15">
       <c r="A20" s="3" t="s">
         <v>58</v>
       </c>
@@ -5894,7 +5894,7 @@
         <v>David Hilton MBE, RN</v>
       </c>
     </row>
-    <row r="21" spans="1:41" ht="15.75" thickBot="1">
+    <row r="21" spans="1:41" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
         <v>60</v>
       </c>
@@ -5982,7 +5982,7 @@
         <v>Paul Thomas Davies</v>
       </c>
     </row>
-    <row r="22" spans="1:41" ht="16.5" thickTop="1" thickBot="1">
+    <row r="22" spans="1:41" ht="16" thickTop="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A22" s="9" t="s">
         <v>63</v>
       </c>
@@ -6068,7 +6068,7 @@
         <v>Michael Graham Fellows</v>
       </c>
     </row>
-    <row r="23" spans="1:41" ht="15.75" thickTop="1">
+    <row r="23" spans="1:41" thickTop="1" x14ac:dyDescent="0.15">
       <c r="A23" s="3" t="s">
         <v>65</v>
       </c>
@@ -6154,7 +6154,7 @@
         <v>Anthony William Latter</v>
       </c>
     </row>
-    <row r="24" spans="1:41">
+    <row r="24" spans="1:41" ht="14" x14ac:dyDescent="0.15">
       <c r="A24" s="3" t="s">
         <v>65</v>
       </c>
@@ -6242,7 +6242,7 @@
         <v>Christopher John Wolohan</v>
       </c>
     </row>
-    <row r="25" spans="1:41">
+    <row r="25" spans="1:41" ht="14" x14ac:dyDescent="0.15">
       <c r="A25" s="3" t="s">
         <v>65</v>
       </c>
@@ -6328,7 +6328,7 @@
         <v>Robert Shane Wilson</v>
       </c>
     </row>
-    <row r="26" spans="1:41">
+    <row r="26" spans="1:41" ht="14" x14ac:dyDescent="0.15">
       <c r="A26" s="3" t="s">
         <v>69</v>
       </c>
@@ -6412,7 +6412,7 @@
         <v>Mark James Legg</v>
       </c>
     </row>
-    <row r="27" spans="1:41">
+    <row r="27" spans="1:41" ht="14" x14ac:dyDescent="0.15">
       <c r="A27" s="3" t="s">
         <v>72</v>
       </c>
@@ -6500,7 +6500,7 @@
         <v>Malcolm James Collier</v>
       </c>
     </row>
-    <row r="28" spans="1:41">
+    <row r="28" spans="1:41" ht="14" x14ac:dyDescent="0.15">
       <c r="A28" s="3" t="s">
         <v>76</v>
       </c>
@@ -6589,7 +6589,7 @@
         <v>David Robert Wood</v>
       </c>
     </row>
-    <row r="29" spans="1:41">
+    <row r="29" spans="1:41" ht="14" x14ac:dyDescent="0.15">
       <c r="A29" s="3" t="s">
         <v>79</v>
       </c>
@@ -6675,7 +6675,7 @@
         <v>Andrew Mark Fuller</v>
       </c>
     </row>
-    <row r="30" spans="1:41">
+    <row r="30" spans="1:41" ht="14" x14ac:dyDescent="0.15">
       <c r="A30" s="3" t="s">
         <v>84</v>
       </c>
@@ -6763,7 +6763,7 @@
         <v>Rodrigo Javier Duarte</v>
       </c>
     </row>
-    <row r="31" spans="1:41">
+    <row r="31" spans="1:41" ht="14" x14ac:dyDescent="0.15">
       <c r="A31" s="3" t="s">
         <v>86</v>
       </c>
@@ -6865,7 +6865,7 @@
         <v>Glyn David Evans</v>
       </c>
     </row>
-    <row r="32" spans="1:41">
+    <row r="32" spans="1:41" ht="14" x14ac:dyDescent="0.15">
       <c r="A32" s="3" t="s">
         <v>90</v>
       </c>
@@ -6956,7 +6956,7 @@
         <v>Philip Andrew Offord</v>
       </c>
     </row>
-    <row r="33" spans="1:51">
+    <row r="33" spans="1:51" ht="14" x14ac:dyDescent="0.15">
       <c r="A33" s="3" t="s">
         <v>92</v>
       </c>
@@ -7042,7 +7042,7 @@
         <v>Alan Vernon Dean</v>
       </c>
     </row>
-    <row r="34" spans="1:51" ht="15.75" thickBot="1">
+    <row r="34" spans="1:51" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
         <v>94</v>
       </c>
@@ -7138,7 +7138,7 @@
       <c r="AX34" s="14"/>
       <c r="AY34" s="14"/>
     </row>
-    <row r="35" spans="1:51" ht="16.5" thickTop="1" thickBot="1">
+    <row r="35" spans="1:51" ht="16" thickTop="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
         <v>96</v>
       </c>
@@ -7234,7 +7234,7 @@
         <v>Thomas Jeremy Ward</v>
       </c>
     </row>
-    <row r="36" spans="1:51" ht="16.5" thickTop="1" thickBot="1">
+    <row r="36" spans="1:51" ht="16" thickTop="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
         <v>96</v>
       </c>
@@ -7320,7 +7320,7 @@
         <v>Gifton Roy Bailey</v>
       </c>
     </row>
-    <row r="37" spans="1:51" ht="16.5" thickTop="1" thickBot="1">
+    <row r="37" spans="1:51" ht="16" thickTop="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A37" s="3" t="s">
         <v>96</v>
       </c>
@@ -7405,7 +7405,7 @@
         <v>Andrew Charles Hodges</v>
       </c>
     </row>
-    <row r="38" spans="1:51" ht="15.75" thickTop="1">
+    <row r="38" spans="1:51" thickTop="1" x14ac:dyDescent="0.15">
       <c r="A38" s="5" t="s">
         <v>96</v>
       </c>
@@ -7485,7 +7485,7 @@
         <v>Carl Jonathan Charles Sams</v>
       </c>
     </row>
-    <row r="39" spans="1:51">
+    <row r="39" spans="1:51" ht="14" x14ac:dyDescent="0.15">
       <c r="A39" s="5" t="s">
         <v>96</v>
       </c>
@@ -7564,7 +7564,7 @@
         <v>John Buck</v>
       </c>
     </row>
-    <row r="40" spans="1:51">
+    <row r="40" spans="1:51" ht="14" x14ac:dyDescent="0.15">
       <c r="A40" s="5" t="s">
         <v>100</v>
       </c>
@@ -7648,7 +7648,7 @@
         <v>Andrew Rhys Morris</v>
       </c>
     </row>
-    <row r="41" spans="1:51">
+    <row r="41" spans="1:51" ht="14" x14ac:dyDescent="0.15">
       <c r="A41" s="5" t="s">
         <v>103</v>
       </c>
@@ -7739,7 +7739,7 @@
         <v>Martin Fields</v>
       </c>
     </row>
-    <row r="42" spans="1:51">
+    <row r="42" spans="1:51" ht="14" x14ac:dyDescent="0.15">
       <c r="A42" s="5" t="s">
         <v>103</v>
       </c>
@@ -7830,7 +7830,7 @@
         <v>Peter Richard Swallow</v>
       </c>
     </row>
-    <row r="43" spans="1:51">
+    <row r="43" spans="1:51" ht="14" x14ac:dyDescent="0.15">
       <c r="A43" s="5" t="s">
         <v>103</v>
       </c>
@@ -7919,7 +7919,7 @@
         <v xml:space="preserve">Anthony Thomas Hill </v>
       </c>
     </row>
-    <row r="44" spans="1:51">
+    <row r="44" spans="1:51" ht="14" x14ac:dyDescent="0.15">
       <c r="A44" s="5" t="s">
         <v>105</v>
       </c>
@@ -8005,7 +8005,7 @@
         <v>Kevin Terence Hutchins</v>
       </c>
     </row>
-    <row r="45" spans="1:51">
+    <row r="45" spans="1:51" ht="14" x14ac:dyDescent="0.15">
       <c r="A45" s="5" t="s">
         <v>108</v>
       </c>
@@ -8095,7 +8095,7 @@
         <v>Jason Michael Curnow</v>
       </c>
     </row>
-    <row r="46" spans="1:51">
+    <row r="46" spans="1:51" ht="14" x14ac:dyDescent="0.15">
       <c r="A46" s="5" t="s">
         <v>108</v>
       </c>
@@ -8181,7 +8181,7 @@
         <v>Neil John White</v>
       </c>
     </row>
-    <row r="47" spans="1:51">
+    <row r="47" spans="1:51" ht="14" x14ac:dyDescent="0.15">
       <c r="A47" s="5" t="s">
         <v>108</v>
       </c>
@@ -8277,7 +8277,7 @@
         <v>James Martin Connolly</v>
       </c>
     </row>
-    <row r="48" spans="1:51">
+    <row r="48" spans="1:51" ht="14" x14ac:dyDescent="0.15">
       <c r="A48" s="5" t="s">
         <v>108</v>
       </c>
@@ -8369,7 +8369,7 @@
         <v>Richard Michael James</v>
       </c>
     </row>
-    <row r="49" spans="1:52">
+    <row r="49" spans="1:52" ht="14" x14ac:dyDescent="0.15">
       <c r="A49" s="5" t="s">
         <v>108</v>
       </c>
@@ -8455,7 +8455,7 @@
         <v>Stephen Mark Abraham</v>
       </c>
     </row>
-    <row r="50" spans="1:52">
+    <row r="50" spans="1:52" ht="14" x14ac:dyDescent="0.15">
       <c r="A50" s="5" t="s">
         <v>108</v>
       </c>
@@ -8543,7 +8543,7 @@
         <v>George David Wilkinson</v>
       </c>
     </row>
-    <row r="51" spans="1:52" ht="15.75" thickBot="1">
+    <row r="51" spans="1:52" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A51" s="5" t="s">
         <v>108</v>
       </c>
@@ -8635,7 +8635,7 @@
         <v>Stephen Paul Madden</v>
       </c>
     </row>
-    <row r="52" spans="1:52" ht="16.5" thickTop="1" thickBot="1">
+    <row r="52" spans="1:52" ht="16" thickTop="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A52" s="5" t="s">
         <v>108</v>
       </c>
@@ -8723,7 +8723,7 @@
         <v>Raymond Hamilton Smith</v>
       </c>
     </row>
-    <row r="53" spans="1:52" ht="15.75" thickTop="1">
+    <row r="53" spans="1:52" thickTop="1" x14ac:dyDescent="0.15">
       <c r="A53" s="5" t="s">
         <v>108</v>
       </c>
@@ -8811,7 +8811,7 @@
         <v>Christopher James Setterfield</v>
       </c>
     </row>
-    <row r="54" spans="1:52">
+    <row r="54" spans="1:52" ht="14" x14ac:dyDescent="0.15">
       <c r="A54" s="68" t="s">
         <v>108</v>
       </c>
@@ -8905,7 +8905,7 @@
         <v>Stephen John Morgan</v>
       </c>
     </row>
-    <row r="55" spans="1:52">
+    <row r="55" spans="1:52" ht="14" x14ac:dyDescent="0.15">
       <c r="A55" s="74" t="s">
         <v>108</v>
       </c>
@@ -8993,7 +8993,7 @@
         <v>Alexander Paul McLennan</v>
       </c>
     </row>
-    <row r="56" spans="1:52">
+    <row r="56" spans="1:52" ht="14" x14ac:dyDescent="0.15">
       <c r="A56" s="74" t="s">
         <v>108</v>
       </c>
@@ -9081,7 +9081,7 @@
         <v>Andrew David Venn</v>
       </c>
     </row>
-    <row r="57" spans="1:52" ht="15" customHeight="1">
+    <row r="57" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A57" s="75" t="s">
         <v>159</v>
       </c>
@@ -9151,7 +9151,7 @@
         <v>Gifton Roy Bailey</v>
       </c>
     </row>
-    <row r="58" spans="1:52" ht="15" customHeight="1">
+    <row r="58" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A58" s="71" t="s">
         <v>160</v>
       </c>
@@ -9225,7 +9225,7 @@
         <v>Thomas Jeremy Ward</v>
       </c>
     </row>
-    <row r="59" spans="1:52" ht="15" customHeight="1">
+    <row r="59" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A59" s="59" t="s">
         <v>161</v>
       </c>
@@ -9301,7 +9301,7 @@
         <v>Michael Geddes</v>
       </c>
     </row>
-    <row r="60" spans="1:52" ht="15" customHeight="1">
+    <row r="60" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A60" s="59" t="s">
         <v>162</v>
       </c>
@@ -9379,7 +9379,7 @@
         <v>Jordan Fretter</v>
       </c>
     </row>
-    <row r="61" spans="1:52" s="28" customFormat="1">
+    <row r="61" spans="1:52" s="28" customFormat="1" ht="14" x14ac:dyDescent="0.15">
       <c r="A61" s="59" t="s">
         <v>163</v>
       </c>
@@ -9452,7 +9452,7 @@
       </c>
       <c r="AZ61" s="12"/>
     </row>
-    <row r="62" spans="1:52" ht="15" customHeight="1">
+    <row r="62" spans="1:52" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A62" s="59" t="s">
         <v>111</v>
       </c>
@@ -9545,19 +9545,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{208D5B5F-72B6-4B46-BC27-C77853048EC1}">
   <dimension ref="D3:S59"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="13.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="4" max="4" width="45.42578125" style="121" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="15.85546875" customWidth="1"/>
-    <col min="13" max="13" width="28.7109375" customWidth="1"/>
-    <col min="14" max="14" width="38.85546875" customWidth="1"/>
-    <col min="16" max="16" width="16.42578125" customWidth="1"/>
-    <col min="17" max="17" width="61.85546875" customWidth="1"/>
+    <col min="4" max="4" width="45.5" style="121" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="15.83203125" customWidth="1"/>
+    <col min="13" max="13" width="28.6640625" customWidth="1"/>
+    <col min="14" max="14" width="38.83203125" customWidth="1"/>
+    <col min="16" max="16" width="16.5" customWidth="1"/>
+    <col min="17" max="17" width="61.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="4:19" ht="30" customHeight="1">
+    <row r="3" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D3" s="123" t="s">
         <v>495</v>
       </c>
@@ -9592,7 +9592,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="4" spans="4:19" ht="30" customHeight="1">
+    <row r="4" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D4" s="210" t="s">
         <v>14</v>
       </c>
@@ -9623,7 +9623,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="5" spans="4:19" ht="30" customHeight="1">
+    <row r="5" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D5" s="210" t="s">
         <v>523</v>
       </c>
@@ -9652,7 +9652,7 @@
       </c>
       <c r="N5" s="115"/>
     </row>
-    <row r="6" spans="4:19" ht="30" customHeight="1">
+    <row r="6" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D6" s="210" t="s">
         <v>524</v>
       </c>
@@ -9686,7 +9686,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="7" spans="4:19" ht="30" customHeight="1">
+    <row r="7" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D7" s="210" t="s">
         <v>115</v>
       </c>
@@ -9717,7 +9717,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="8" spans="4:19" ht="30" customHeight="1">
+    <row r="8" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D8" s="210" t="s">
         <v>36</v>
       </c>
@@ -9746,7 +9746,7 @@
       </c>
       <c r="N8" s="115"/>
     </row>
-    <row r="9" spans="4:19" ht="30" customHeight="1">
+    <row r="9" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D9" s="118" t="s">
         <v>41</v>
       </c>
@@ -9777,7 +9777,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="10" spans="4:19" ht="30" customHeight="1">
+    <row r="10" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D10" s="148" t="s">
         <v>46</v>
       </c>
@@ -9817,7 +9817,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="11" spans="4:19" ht="30" customHeight="1">
+    <row r="11" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D11" s="151" t="s">
         <v>48</v>
       </c>
@@ -9856,7 +9856,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="12" spans="4:19" ht="30" customHeight="1">
+    <row r="12" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D12" s="119" t="s">
         <v>52</v>
       </c>
@@ -9893,7 +9893,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="13" spans="4:19" ht="30" customHeight="1">
+    <row r="13" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D13" s="119" t="s">
         <v>55</v>
       </c>
@@ -9932,7 +9932,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="14" spans="4:19" ht="30" customHeight="1">
+    <row r="14" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D14" s="119" t="s">
         <v>58</v>
       </c>
@@ -9973,7 +9973,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="15" spans="4:19" ht="30" customHeight="1">
+    <row r="15" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D15" s="119" t="s">
         <v>60</v>
       </c>
@@ -10004,7 +10004,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="16" spans="4:19" ht="30" customHeight="1">
+    <row r="16" spans="4:19" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D16" s="154" t="s">
         <v>63</v>
       </c>
@@ -10037,7 +10037,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="17" spans="4:16" ht="30" customHeight="1">
+    <row r="17" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D17" s="119" t="s">
         <v>65</v>
       </c>
@@ -10070,7 +10070,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="18" spans="4:16" ht="30" customHeight="1">
+    <row r="18" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D18" s="119" t="s">
         <v>65</v>
       </c>
@@ -10101,7 +10101,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="19" spans="4:16" ht="30" customHeight="1">
+    <row r="19" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D19" s="119" t="s">
         <v>65</v>
       </c>
@@ -10134,7 +10134,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="20" spans="4:16" ht="30" customHeight="1">
+    <row r="20" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D20" s="119" t="s">
         <v>69</v>
       </c>
@@ -10167,7 +10167,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="21" spans="4:16" ht="30" customHeight="1">
+    <row r="21" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D21" s="119" t="s">
         <v>72</v>
       </c>
@@ -10200,7 +10200,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="22" spans="4:16" ht="30" customHeight="1">
+    <row r="22" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D22" s="119" t="s">
         <v>76</v>
       </c>
@@ -10236,7 +10236,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="23" spans="4:16" ht="30" customHeight="1">
+    <row r="23" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D23" s="119" t="s">
         <v>79</v>
       </c>
@@ -10267,7 +10267,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="24" spans="4:16" ht="30" customHeight="1">
+    <row r="24" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D24" s="119" t="s">
         <v>84</v>
       </c>
@@ -10298,7 +10298,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="25" spans="4:16" ht="30" customHeight="1">
+    <row r="25" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D25" s="119" t="s">
         <v>86</v>
       </c>
@@ -10334,7 +10334,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="26" spans="4:16" ht="30" customHeight="1">
+    <row r="26" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D26" s="119" t="s">
         <v>90</v>
       </c>
@@ -10367,7 +10367,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="27" spans="4:16" ht="30" customHeight="1">
+    <row r="27" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D27" s="119" t="s">
         <v>92</v>
       </c>
@@ -10398,7 +10398,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="28" spans="4:16" ht="30" customHeight="1">
+    <row r="28" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D28" s="155" t="s">
         <v>94</v>
       </c>
@@ -10431,7 +10431,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="29" spans="4:16" ht="30" customHeight="1">
+    <row r="29" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D29" s="158" t="s">
         <v>96</v>
       </c>
@@ -10464,7 +10464,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="30" spans="4:16" ht="30" customHeight="1">
+    <row r="30" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D30" s="119" t="s">
         <v>96</v>
       </c>
@@ -10495,7 +10495,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="31" spans="4:16" ht="30" customHeight="1">
+    <row r="31" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D31" s="155" t="s">
         <v>96</v>
       </c>
@@ -10526,7 +10526,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="32" spans="4:16" ht="30" customHeight="1">
+    <row r="32" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D32" s="161" t="s">
         <v>96</v>
       </c>
@@ -10559,7 +10559,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="33" spans="4:16" ht="30" customHeight="1">
+    <row r="33" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D33" s="124" t="s">
         <v>96</v>
       </c>
@@ -10592,7 +10592,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="34" spans="4:16" ht="30" customHeight="1">
+    <row r="34" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D34" s="124" t="s">
         <v>100</v>
       </c>
@@ -10625,7 +10625,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="35" spans="4:16" ht="30" customHeight="1">
+    <row r="35" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D35" s="162" t="s">
         <v>103</v>
       </c>
@@ -10658,7 +10658,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="36" spans="4:16" ht="30" customHeight="1">
+    <row r="36" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D36" s="124" t="s">
         <v>103</v>
       </c>
@@ -10691,7 +10691,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="37" spans="4:16" ht="30" customHeight="1">
+    <row r="37" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D37" s="163" t="s">
         <v>103</v>
       </c>
@@ -10724,7 +10724,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="38" spans="4:16" ht="30" customHeight="1">
+    <row r="38" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D38" s="124" t="s">
         <v>105</v>
       </c>
@@ -10757,7 +10757,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="39" spans="4:16" ht="30" customHeight="1">
+    <row r="39" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D39" s="164" t="s">
         <v>108</v>
       </c>
@@ -10790,7 +10790,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="40" spans="4:16" ht="30" customHeight="1">
+    <row r="40" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D40" s="161" t="s">
         <v>108</v>
       </c>
@@ -10823,7 +10823,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="41" spans="4:16" ht="30" customHeight="1">
+    <row r="41" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D41" s="162" t="s">
         <v>108</v>
       </c>
@@ -10857,7 +10857,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="42" spans="4:16" ht="30" customHeight="1">
+    <row r="42" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D42" s="162" t="s">
         <v>108</v>
       </c>
@@ -10890,7 +10890,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="43" spans="4:16" ht="30" customHeight="1">
+    <row r="43" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D43" s="168" t="s">
         <v>108</v>
       </c>
@@ -10923,7 +10923,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="44" spans="4:16" ht="30" customHeight="1">
+    <row r="44" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D44" s="162" t="s">
         <v>108</v>
       </c>
@@ -10959,7 +10959,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="45" spans="4:16" ht="30" customHeight="1">
+    <row r="45" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D45" s="161" t="s">
         <v>108</v>
       </c>
@@ -10990,7 +10990,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="46" spans="4:16" ht="30" customHeight="1">
+    <row r="46" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D46" s="161" t="s">
         <v>108</v>
       </c>
@@ -11026,7 +11026,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="47" spans="4:16" ht="30" customHeight="1">
+    <row r="47" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D47" s="124" t="s">
         <v>108</v>
       </c>
@@ -11059,7 +11059,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="48" spans="4:16" ht="30" customHeight="1">
+    <row r="48" spans="4:16" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D48" s="124" t="s">
         <v>108</v>
       </c>
@@ -11092,7 +11092,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="49" spans="4:14" ht="30" customHeight="1">
+    <row r="49" spans="4:14" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D49" s="122" t="s">
         <v>108</v>
       </c>
@@ -11121,7 +11121,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="50" spans="4:14" ht="30" customHeight="1">
+    <row r="50" spans="4:14" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D50" s="189" t="s">
         <v>108</v>
       </c>
@@ -11154,7 +11154,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="51" spans="4:14">
+    <row r="51" spans="4:14" ht="15" x14ac:dyDescent="0.15">
       <c r="D51" s="215" t="s">
         <v>560</v>
       </c>
@@ -11179,7 +11179,7 @@
       </c>
       <c r="N51" s="216"/>
     </row>
-    <row r="52" spans="4:14">
+    <row r="52" spans="4:14" ht="15" x14ac:dyDescent="0.15">
       <c r="D52" s="215" t="s">
         <v>564</v>
       </c>
@@ -11204,7 +11204,7 @@
       </c>
       <c r="N52" s="216"/>
     </row>
-    <row r="53" spans="4:14">
+    <row r="53" spans="4:14" ht="15" x14ac:dyDescent="0.15">
       <c r="D53" s="215" t="s">
         <v>566</v>
       </c>
@@ -11229,7 +11229,7 @@
       </c>
       <c r="N53" s="216"/>
     </row>
-    <row r="54" spans="4:14">
+    <row r="54" spans="4:14" x14ac:dyDescent="0.15">
       <c r="E54" s="114"/>
       <c r="F54" s="114"/>
       <c r="G54" s="114"/>
@@ -11241,7 +11241,7 @@
       <c r="M54" s="114"/>
       <c r="N54" s="114"/>
     </row>
-    <row r="55" spans="4:14">
+    <row r="55" spans="4:14" x14ac:dyDescent="0.15">
       <c r="E55" s="114"/>
       <c r="F55" s="114"/>
       <c r="G55" s="114"/>
@@ -11253,7 +11253,7 @@
       <c r="M55" s="114"/>
       <c r="N55" s="114"/>
     </row>
-    <row r="56" spans="4:14">
+    <row r="56" spans="4:14" x14ac:dyDescent="0.15">
       <c r="E56" s="114"/>
       <c r="F56" s="114"/>
       <c r="G56" s="114"/>
@@ -11265,7 +11265,7 @@
       <c r="M56" s="114"/>
       <c r="N56" s="114"/>
     </row>
-    <row r="57" spans="4:14">
+    <row r="57" spans="4:14" x14ac:dyDescent="0.15">
       <c r="E57" s="114"/>
       <c r="F57" s="114"/>
       <c r="G57" s="114"/>
@@ -11277,7 +11277,7 @@
       <c r="M57" s="114"/>
       <c r="N57" s="114"/>
     </row>
-    <row r="58" spans="4:14">
+    <row r="58" spans="4:14" x14ac:dyDescent="0.15">
       <c r="E58" s="114"/>
       <c r="F58" s="114"/>
       <c r="G58" s="114"/>
@@ -11289,7 +11289,7 @@
       <c r="M58" s="114"/>
       <c r="N58" s="114"/>
     </row>
-    <row r="59" spans="4:14">
+    <row r="59" spans="4:14" x14ac:dyDescent="0.15">
       <c r="E59" s="114"/>
       <c r="F59" s="114"/>
       <c r="G59" s="114"/>

</xml_diff>